<commit_message>
added remy and updated schedule
</commit_message>
<xml_diff>
--- a/admin/Schedule.xlsx
+++ b/admin/Schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USER-PC\Ravens\Ravens2026Juniors\tournament manager\admin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913CDED5-6F3F-4B37-932A-347EADCC7FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD5D5B7-4E5F-4BC1-B9F2-C8DE78EEF239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83DAA105-BFF5-46A2-B12A-FB59EB91345B}"/>
+    <workbookView xWindow="6240" yWindow="2175" windowWidth="20370" windowHeight="10770" xr2:uid="{83DAA105-BFF5-46A2-B12A-FB59EB91345B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="62">
   <si>
     <t>u15 Girls Group 1</t>
   </si>
@@ -665,10 +665,10 @@
         <v>2</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -685,19 +685,19 @@
         <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -755,7 +755,7 @@
         <v>4</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -780,11 +780,8 @@
       <c r="G6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="I6" s="1" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -809,6 +806,9 @@
       <c r="G7" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="H7" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="I7" s="1" t="s">
         <v>23</v>
       </c>
@@ -835,6 +835,9 @@
       <c r="G8" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="H8" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="I8" s="1" t="s">
         <v>23</v>
       </c>
@@ -907,14 +910,16 @@
         <v>48</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>